<commit_message>
Enhance user interface in app.py by hiding the theme selection menu and fixing the default theme to Light. Update README.md to include troubleshooting tips and clarify installation instructions. Improve filename parsing in data_load_mode.py and general_analysis_mode.py to auto-fill enzyme and substrate names based on uploaded file names. Update Excel files for consistency in data representation.
</commit_message>
<xml_diff>
--- a/ref/260305_protease_conc_time_YL.xlsx
+++ b/ref/260305_protease_conc_time_YL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sookmyungackr-my.sharepoint.com/personal/yul_sookmyung_ac_kr/Documents/문서/YL/2. BSL/1. Works/5. 구강세균/실험 결과/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\hyacinth1126\protease-simulator-3\ref\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{E0F01A36-AE37-4B6A-AAB4-29D53FA0550D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AF358FD-B1B5-479F-AA34-167FF95C323F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{942BD6BE-4203-4B4D-A2E4-3DB738781A0C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26130" yWindow="165" windowWidth="25590" windowHeight="14280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26130" yWindow="165" windowWidth="25590" windowHeight="14280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kgp sensor" sheetId="1" r:id="rId1"/>
@@ -22,23 +22,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="22">
   <si>
     <t>RFU</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -104,6 +93,22 @@
   </si>
   <si>
     <t>- Add 10 ul peptide solution to the hydrogel and incubate for 2 h.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Kgp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>kDa</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RgpA</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RgpB</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -192,13 +197,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -223,15 +228,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>2485</xdr:colOff>
+          <xdr:colOff>0</xdr:colOff>
           <xdr:row>12</xdr:row>
-          <xdr:rowOff>198783</xdr:rowOff>
+          <xdr:rowOff>200025</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>4</xdr:col>
-          <xdr:colOff>770282</xdr:colOff>
+          <xdr:colOff>771525</xdr:colOff>
           <xdr:row>17</xdr:row>
-          <xdr:rowOff>182218</xdr:rowOff>
+          <xdr:rowOff>180975</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -296,7 +301,7 @@
         <xdr:cNvPr id="2" name="그림 1" descr="스크린샷이(가) 표시된 사진&#10;&#10;AI 생성 콘텐츠는 정확하지 않을 수 있습니다.">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F9646C2C-55DB-1465-8E02-3ABBF44FD758}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -352,7 +357,7 @@
         <xdr:cNvPr id="2" name="그림 1" descr="스크린샷이(가) 표시된 사진&#10;&#10;AI 생성 콘텐츠는 정확하지 않을 수 있습니다.">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9A4BBE52-A252-4CCB-552D-9D6A84507501}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -651,7 +656,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="3.75" customWidth="1"/>
@@ -662,35 +667,35 @@
     <row r="1" spans="1:15" ht="11.25" customHeight="1"/>
     <row r="2" spans="1:15" s="1" customFormat="1" ht="18" customHeight="1">
       <c r="A2"/>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4" t="s">
+      <c r="D2" s="5"/>
+      <c r="E2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4" t="s">
+      <c r="F2" s="5"/>
+      <c r="G2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4" t="s">
+      <c r="H2" s="5"/>
+      <c r="I2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4" t="s">
+      <c r="J2" s="5"/>
+      <c r="K2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L2" s="4"/>
+      <c r="L2" s="5"/>
       <c r="M2"/>
       <c r="N2"/>
       <c r="O2"/>
     </row>
     <row r="3" spans="1:15">
-      <c r="B3" s="5"/>
+      <c r="B3" s="6"/>
       <c r="C3" s="2" t="s">
         <v>0</v>
       </c>
@@ -1002,19 +1007,30 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="3:6">
+    <row r="17" spans="2:6">
       <c r="F17" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="3:6">
+    <row r="18" spans="2:6">
       <c r="F18" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="3:6">
+    <row r="19" spans="2:6">
       <c r="C19" s="3" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6">
+      <c r="B22" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22">
+        <v>56.6</v>
+      </c>
+      <c r="D22" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1028,13 +1044,14 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
   <oleObjects>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <oleObject progId="ChemDraw.Document.6.0" shapeId="1025" r:id="rId3">
-          <objectPr defaultSize="0" autoPict="0" r:id="rId4">
+        <oleObject progId="ChemDraw.Document.6.0" shapeId="1025" r:id="rId4">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId5">
             <anchor moveWithCells="1">
               <from>
                 <xdr:col>2</xdr:col>
@@ -1053,7 +1070,7 @@
         </oleObject>
       </mc:Choice>
       <mc:Fallback>
-        <oleObject progId="ChemDraw.Document.6.0" shapeId="1025" r:id="rId3"/>
+        <oleObject progId="ChemDraw.Document.6.0" shapeId="1025" r:id="rId4"/>
       </mc:Fallback>
     </mc:AlternateContent>
   </oleObjects>
@@ -1062,7 +1079,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{907AA74A-AD95-487C-9D66-67686C8B8366}">
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="3.75" customWidth="1"/>
@@ -1073,35 +1090,35 @@
     <row r="1" spans="1:15" ht="11.25" customHeight="1"/>
     <row r="2" spans="1:15" s="1" customFormat="1" ht="18" customHeight="1">
       <c r="A2"/>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4" t="s">
+      <c r="D2" s="5"/>
+      <c r="E2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4" t="s">
+      <c r="F2" s="5"/>
+      <c r="G2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4" t="s">
+      <c r="H2" s="5"/>
+      <c r="I2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4" t="s">
+      <c r="J2" s="5"/>
+      <c r="K2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L2" s="4"/>
+      <c r="L2" s="5"/>
       <c r="M2"/>
       <c r="N2"/>
       <c r="O2"/>
     </row>
     <row r="3" spans="1:15">
-      <c r="B3" s="5"/>
+      <c r="B3" s="6"/>
       <c r="C3" s="2" t="s">
         <v>0</v>
       </c>
@@ -1157,34 +1174,34 @@
       <c r="B5">
         <v>1</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="4">
         <v>2401.5700000000002</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="4">
         <v>125.999</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="4">
         <v>3659.89</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="4">
         <v>692.76800000000003</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="4">
         <v>4472.7299999999996</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="4">
         <v>135.48599999999999</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="4">
         <v>8464.61</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="4">
         <v>262.75799999999998</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="4">
         <v>11134.53</v>
       </c>
-      <c r="L5" s="6">
+      <c r="L5" s="4">
         <v>591.31799999999998</v>
       </c>
     </row>
@@ -1192,34 +1209,34 @@
       <c r="B6">
         <v>5</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="4">
         <v>3093.45</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <v>105.11199999999999</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="4">
         <v>4150.32</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="4">
         <v>550.56700000000001</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="4">
         <v>6460.81</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="4">
         <v>498.01900000000001</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="4">
         <v>8603.99</v>
       </c>
-      <c r="J6" s="6">
+      <c r="J6" s="4">
         <v>515.01099999999997</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="4">
         <v>11265.1</v>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="4">
         <v>385.08800000000002</v>
       </c>
     </row>
@@ -1227,34 +1244,34 @@
       <c r="B7">
         <v>10</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="4">
         <v>4129.92</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="4">
         <v>393.48500000000001</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="4">
         <v>6040.28</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="4">
         <v>216.29499999999999</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="4">
         <v>7752.69</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="4">
         <v>642.47199999999998</v>
       </c>
-      <c r="I7" s="6">
+      <c r="I7" s="4">
         <v>8638.7800000000007</v>
       </c>
-      <c r="J7" s="6">
+      <c r="J7" s="4">
         <v>365.47800000000001</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="4">
         <v>11284.1</v>
       </c>
-      <c r="L7" s="6">
+      <c r="L7" s="4">
         <v>559.16</v>
       </c>
     </row>
@@ -1262,34 +1279,34 @@
       <c r="B8">
         <v>15</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="4">
         <v>4955.8500000000004</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="4">
         <v>110.155</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="4">
         <v>7248.42</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="4">
         <v>155.12200000000001</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="4">
         <v>8303.3799999999992</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="4">
         <v>160.23099999999999</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="4">
         <v>9502.81</v>
       </c>
-      <c r="J8" s="6">
+      <c r="J8" s="4">
         <v>175.244</v>
       </c>
-      <c r="K8" s="6">
+      <c r="K8" s="4">
         <v>11848.43</v>
       </c>
-      <c r="L8" s="6">
+      <c r="L8" s="4">
         <v>375.291</v>
       </c>
     </row>
@@ -1297,34 +1314,34 @@
       <c r="B9">
         <v>20</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="4">
         <v>5203.7700000000004</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="4">
         <v>483.72199999999998</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="4">
         <v>7610.78</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="4">
         <v>295.31099999999998</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="4">
         <v>8768.5499999999993</v>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="4">
         <v>373.43</v>
       </c>
-      <c r="I9" s="6">
+      <c r="I9" s="4">
         <v>9937.2199999999993</v>
       </c>
-      <c r="J9" s="6">
+      <c r="J9" s="4">
         <v>621.50099999999998</v>
       </c>
-      <c r="K9" s="6">
+      <c r="K9" s="4">
         <v>11966.95</v>
       </c>
-      <c r="L9" s="6">
+      <c r="L9" s="4">
         <v>280.55200000000002</v>
       </c>
     </row>
@@ -1332,34 +1349,34 @@
       <c r="B10">
         <v>25</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="4">
         <v>4943.59</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="4">
         <v>113.92100000000001</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="4">
         <v>7229.83</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="4">
         <v>355.452</v>
       </c>
-      <c r="G10" s="6">
+      <c r="G10" s="4">
         <v>9023.1200000000008</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="4">
         <v>375.601</v>
       </c>
-      <c r="I10" s="6">
+      <c r="I10" s="4">
         <v>9588.33</v>
       </c>
-      <c r="J10" s="6">
+      <c r="J10" s="4">
         <v>460.71100000000001</v>
       </c>
-      <c r="K10" s="6">
+      <c r="K10" s="4">
         <v>11727.63</v>
       </c>
-      <c r="L10" s="6">
+      <c r="L10" s="4">
         <v>185.792</v>
       </c>
     </row>
@@ -1367,34 +1384,34 @@
       <c r="B11">
         <v>30</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="4">
         <v>4449.2700000000004</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="4">
         <v>296.07499999999999</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="4">
         <v>6506.89</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="4">
         <v>100.589</v>
       </c>
-      <c r="G11" s="6">
+      <c r="G11" s="4">
         <v>8352.2800000000007</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="4">
         <v>280.887</v>
       </c>
-      <c r="I11" s="6">
+      <c r="I11" s="4">
         <v>9137.89</v>
       </c>
-      <c r="J11" s="6">
+      <c r="J11" s="4">
         <v>195.9</v>
       </c>
-      <c r="K11" s="6">
+      <c r="K11" s="4">
         <v>11140.25</v>
       </c>
-      <c r="L11" s="6">
+      <c r="L11" s="4">
         <v>490.91</v>
       </c>
     </row>
@@ -1413,29 +1430,40 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="3:6">
+    <row r="17" spans="2:6">
       <c r="F17" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="3:6">
+    <row r="18" spans="2:6">
       <c r="F18" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="3:6">
+    <row r="20" spans="2:6">
       <c r="C20" s="3" t="s">
         <v>14</v>
       </c>
     </row>
+    <row r="22" spans="2:6">
+      <c r="B22" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22">
+        <v>56</v>
+      </c>
+      <c r="D22" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="K2:L2"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="K2:L2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1446,7 +1474,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{520ECB33-7656-4F87-B5E1-6725EFEB385B}">
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="3.75" customWidth="1"/>
@@ -1457,35 +1485,35 @@
     <row r="1" spans="1:15" ht="11.25" customHeight="1"/>
     <row r="2" spans="1:15" s="1" customFormat="1" ht="18" customHeight="1">
       <c r="A2"/>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4" t="s">
+      <c r="D2" s="5"/>
+      <c r="E2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4" t="s">
+      <c r="F2" s="5"/>
+      <c r="G2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4" t="s">
+      <c r="H2" s="5"/>
+      <c r="I2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4" t="s">
+      <c r="J2" s="5"/>
+      <c r="K2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L2" s="4"/>
+      <c r="L2" s="5"/>
       <c r="M2"/>
       <c r="N2"/>
       <c r="O2"/>
     </row>
     <row r="3" spans="1:15">
-      <c r="B3" s="5"/>
+      <c r="B3" s="6"/>
       <c r="C3" s="2" t="s">
         <v>0</v>
       </c>
@@ -1541,34 +1569,34 @@
       <c r="B5">
         <v>1</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="4">
         <v>2401.54</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="4">
         <v>125.209</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="4">
         <v>3340.46</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="4">
         <v>479.767</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="4">
         <v>5472.33</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="4">
         <v>155.48599999999999</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="4">
         <v>8464.61</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="4">
         <v>462.75760000000002</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="4">
         <v>11134.64</v>
       </c>
-      <c r="L5" s="6">
+      <c r="L5" s="4">
         <v>391.31700000000001</v>
       </c>
     </row>
@@ -1576,34 +1604,34 @@
       <c r="B6">
         <v>5</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="4">
         <v>3110.41</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <v>514.98699999999997</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="4">
         <v>5005.67</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="4">
         <v>154.90199999999999</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="4">
         <v>8155.85</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="4">
         <v>463.351</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="4">
         <v>10005.370000000001</v>
       </c>
-      <c r="J6" s="6">
+      <c r="J6" s="4">
         <v>556.55930000000001</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="4">
         <v>13405.17</v>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="4">
         <v>466.44600000000003</v>
       </c>
     </row>
@@ -1611,34 +1639,34 @@
       <c r="B7">
         <v>10</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="4">
         <v>3840.81</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="4">
         <v>408.565</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="4">
         <v>6380.12</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="4">
         <v>346.82</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="4">
         <v>9855.02</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="4">
         <v>560.60299999999995</v>
       </c>
-      <c r="I7" s="6">
+      <c r="I7" s="4">
         <v>12805.65</v>
       </c>
-      <c r="J7" s="6">
+      <c r="J7" s="4">
         <v>522.65899999999999</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="4">
         <v>14850.84</v>
       </c>
-      <c r="L7" s="6">
+      <c r="L7" s="4">
         <v>283.93099999999998</v>
       </c>
     </row>
@@ -1646,34 +1674,34 @@
       <c r="B8">
         <v>15</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="4">
         <v>4571.16</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="4">
         <v>122.28</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="4">
         <v>7664.65</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="4">
         <v>159.833</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="4">
         <v>12503.25</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="4">
         <v>201.21799999999999</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="4">
         <v>14550.43</v>
       </c>
-      <c r="J8" s="6">
+      <c r="J8" s="4">
         <v>462.37099999999998</v>
       </c>
-      <c r="K8" s="6">
+      <c r="K8" s="4">
         <v>15917.09</v>
       </c>
-      <c r="L8" s="6">
+      <c r="L8" s="4">
         <v>458.762</v>
       </c>
     </row>
@@ -1681,34 +1709,34 @@
       <c r="B9">
         <v>20</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="4">
         <v>4250.3500000000004</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="4">
         <v>507.404</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="4">
         <v>7350.44</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="4">
         <v>414.13600000000002</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="4">
         <v>11880.82</v>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="4">
         <v>291.82600000000002</v>
       </c>
-      <c r="I9" s="6">
+      <c r="I9" s="4">
         <v>14155.29</v>
       </c>
-      <c r="J9" s="6">
+      <c r="J9" s="4">
         <v>316.46899999999999</v>
       </c>
-      <c r="K9" s="6">
+      <c r="K9" s="4">
         <v>16015.35</v>
       </c>
-      <c r="L9" s="6">
+      <c r="L9" s="4">
         <v>199.72200000000001</v>
       </c>
     </row>
@@ -1716,34 +1744,34 @@
       <c r="B10">
         <v>25</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="4">
         <v>4605.82</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="4">
         <v>379.40699999999998</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="4">
         <v>7135.19</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="4">
         <v>527.40200000000004</v>
       </c>
-      <c r="G10" s="6">
+      <c r="G10" s="4">
         <v>12050.47</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="4">
         <v>356.95</v>
       </c>
-      <c r="I10" s="6">
+      <c r="I10" s="4">
         <v>13850.93</v>
       </c>
-      <c r="J10" s="6">
+      <c r="J10" s="4">
         <v>525.58399999999995</v>
       </c>
-      <c r="K10" s="6">
+      <c r="K10" s="4">
         <v>15855.96</v>
       </c>
-      <c r="L10" s="6">
+      <c r="L10" s="4">
         <v>547.94299999999998</v>
       </c>
     </row>
@@ -1751,34 +1779,34 @@
       <c r="B11">
         <v>30</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="4">
         <v>4001.45</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="4">
         <v>264.20299999999997</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="4">
         <v>7390.62</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="4">
         <v>375.54199999999997</v>
       </c>
-      <c r="G11" s="6">
+      <c r="G11" s="4">
         <v>12080.31</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="4">
         <v>181.02600000000001</v>
       </c>
-      <c r="I11" s="6">
+      <c r="I11" s="4">
         <v>13505.47</v>
       </c>
-      <c r="J11" s="6">
+      <c r="J11" s="4">
         <v>243.70400000000001</v>
       </c>
-      <c r="K11" s="6">
+      <c r="K11" s="4">
         <v>15050.62</v>
       </c>
-      <c r="L11" s="6">
+      <c r="L11" s="4">
         <v>572.51</v>
       </c>
     </row>
@@ -1797,29 +1825,40 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="3:6">
+    <row r="17" spans="2:6">
       <c r="F17" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="3:6">
+    <row r="18" spans="2:6">
       <c r="F18" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="3:6">
+    <row r="20" spans="2:6">
       <c r="C20" s="3" t="s">
         <v>15</v>
       </c>
     </row>
+    <row r="22" spans="2:6">
+      <c r="B22" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22">
+        <v>43.3</v>
+      </c>
+      <c r="D22" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="K2:L2"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="K2:L2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>